<commit_message>
Cambio de 375 a formato ET
</commit_message>
<xml_diff>
--- a/public/ET.xlsx
+++ b/public/ET.xlsx
@@ -173,10 +173,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>